<commit_message>
fix: 3rd testing round fixes
</commit_message>
<xml_diff>
--- a/issue_classification_master.xlsx
+++ b/issue_classification_master.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +61,21 @@
       <b val="1"/>
       <color rgb="009C6500"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +110,26 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
         <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -234,6 +267,21 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -608,9 +656,10 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -639,6 +688,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>Reason / Notes</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2788,711 @@
       <c r="E70" s="22" t="n"/>
       <c r="F70" s="21" t="n"/>
     </row>
+    <row r="71">
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>3rd Round — Heat-Cool Portal Improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>IMP-05</t>
+        </is>
+      </c>
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C72" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E72" s="24" t="inlineStr">
+        <is>
+          <t>Mandatory fields in the 'Add Staff' form are not clearly marked with required indicators.</t>
+        </is>
+      </c>
+      <c r="F72" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>IMP-13</t>
+        </is>
+      </c>
+      <c r="B73" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E73" s="24" t="inlineStr">
+        <is>
+          <t>The current active page does not highlight when the user opens the building details page.</t>
+        </is>
+      </c>
+      <c r="F73" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>IMP-14</t>
+        </is>
+      </c>
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C74" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="inlineStr">
+        <is>
+          <t>Missing 'x' button on the 'Upload Utility &amp; Degree Day Data' pop-up.</t>
+        </is>
+      </c>
+      <c r="F74" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>IMP-15</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>Total kBTU field remains editable after being auto-calculated from fuel fields; should be read-only when auto-calculated.</t>
+        </is>
+      </c>
+      <c r="F75" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>IMP-19</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C76" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E76" s="24" t="inlineStr">
+        <is>
+          <t>The cursor icon changes to a hand pointer on disabled buttons.</t>
+        </is>
+      </c>
+      <c r="F76" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="24" t="inlineStr">
+        <is>
+          <t>IMP-22</t>
+        </is>
+      </c>
+      <c r="B77" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E77" s="24" t="inlineStr">
+        <is>
+          <t>The cursor icon changes to a hand pointer on disabled buttons in the Building portal Recent Messages section.</t>
+        </is>
+      </c>
+      <c r="F77" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>IMP-01</t>
+        </is>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E78" s="24" t="inlineStr">
+        <is>
+          <t>Dashboard summary cards (Total Cities, Active Buildings, Alert Logs, Compliance Rate) are not interactive and not linked to their respective sections.</t>
+        </is>
+      </c>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="28" t="inlineStr">
+        <is>
+          <t>IMP-02</t>
+        </is>
+      </c>
+      <c r="B79" s="28" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C79" s="28" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D79" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E79" s="28" t="inlineStr">
+        <is>
+          <t>Daily summary includes invalid, duplicate, and out-of-scope city names (e.g., incomplete names, random strings, non-northeast cities).</t>
+        </is>
+      </c>
+      <c r="F79" s="29" t="inlineStr">
+        <is>
+          <t>N/A – Data Issue</t>
+        </is>
+      </c>
+      <c r="G79" s="30" t="inlineStr">
+        <is>
+          <t>City names appear invalid/duplicated because of test/bad data entered into the system. The code correctly displays what is stored — this is a data quality issue, not a code bug. Fix: clean up the city data in the database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="28" t="inlineStr">
+        <is>
+          <t>IMP-03</t>
+        </is>
+      </c>
+      <c r="B80" s="28" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C80" s="28" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D80" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E80" s="28" t="inlineStr">
+        <is>
+          <t>Alert IDs are returned separately from city and alert metadata, making it impossible to trace which ID belongs to which alert condition.</t>
+        </is>
+      </c>
+      <c r="F80" s="29" t="inlineStr">
+        <is>
+          <t>N/A – By Design</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="inlineStr">
+        <is>
+          <t>The 'Check Alerts' trigger output is generated by the Message Triggers panel, which is an admin developer tool used to manually run cron jobs. It is not a user-facing feature. The raw API response format is intentional for debugging purposes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E81" s="24" t="inlineStr">
+        <is>
+          <t>Message triggers (system outputs) are displayed in raw JSON format instead of a user-friendly representation.</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="25" t="inlineStr">
+        <is>
+          <t>IMP-06</t>
+        </is>
+      </c>
+      <c r="B82" s="25" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C82" s="25" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D82" s="25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E82" s="25" t="inlineStr">
+        <is>
+          <t>Buildings created in the Admin portal are not reflected in the Building portal interface.</t>
+        </is>
+      </c>
+      <c r="F82" s="25" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="28" t="inlineStr">
+        <is>
+          <t>IMP-07</t>
+        </is>
+      </c>
+      <c r="B83" s="28" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C83" s="28" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D83" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E83" s="28" t="inlineStr">
+        <is>
+          <t>Alerts displayed in the system are not interactive and lack clear explanation or context.</t>
+        </is>
+      </c>
+      <c r="F83" s="29" t="inlineStr">
+        <is>
+          <t>N/A – By Design</t>
+        </is>
+      </c>
+      <c r="G83" s="30" t="inlineStr">
+        <is>
+          <t>The Building portal is intentionally read-only (the footer states: 'View-only access. This portal provides read-only access to your building's data.'). Alerts are informational only; management is handled via the Admin portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>IMP-08</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>System does not clearly indicate when a user lacks permission to view uploads.</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="31" t="inlineStr">
+        <is>
+          <t>IMP-09</t>
+        </is>
+      </c>
+      <c r="B85" s="31" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C85" s="31" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D85" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E85" s="31" t="inlineStr">
+        <is>
+          <t>Uploaded files are not accessible or visible after submission.</t>
+        </is>
+      </c>
+      <c r="F85" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G85" s="31" t="inlineStr">
+        <is>
+          <t>UX fix: success message lists processed months/years + auto-scroll to utility history table after Excel upload. Staff can see data immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="24" t="inlineStr">
+        <is>
+          <t>IMP-10</t>
+        </is>
+      </c>
+      <c r="B86" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C86" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D86" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>System throws an error when uploading bulk data through Excel even when data is correct.</t>
+        </is>
+      </c>
+      <c r="F86" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="25" t="inlineStr">
+        <is>
+          <t>IMP-11</t>
+        </is>
+      </c>
+      <c r="B87" s="25" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="D87" s="25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E87" s="25" t="inlineStr">
+        <is>
+          <t>Energy saving reports are presented in a basic and unstructured format without charts or visual hierarchy.</t>
+        </is>
+      </c>
+      <c r="F87" s="25" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="24" t="inlineStr">
+        <is>
+          <t>IMP-16</t>
+        </is>
+      </c>
+      <c r="B88" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D88" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E88" s="24" t="inlineStr">
+        <is>
+          <t>The utility bill appears on the staff end but does not appear on the Admin's building details page.</t>
+        </is>
+      </c>
+      <c r="F88" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="24" t="inlineStr">
+        <is>
+          <t>IMP-17</t>
+        </is>
+      </c>
+      <c r="B89" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E89" s="24" t="inlineStr">
+        <is>
+          <t>Paused building status is not reflected on staff end; staff can still add utility bill and generate reports for paused buildings.</t>
+        </is>
+      </c>
+      <c r="F89" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>IMP-18</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D90" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>Deactivated building is still accessible to staff and building users who can add utility data and generate reports.</t>
+        </is>
+      </c>
+      <c r="F90" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="24" t="inlineStr">
+        <is>
+          <t>IMP-20</t>
+        </is>
+      </c>
+      <c r="B91" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C91" s="24" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="D91" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E91" s="24" t="inlineStr">
+        <is>
+          <t>Missing sorting functionality for the buildings table on the Admin portal.</t>
+        </is>
+      </c>
+      <c r="F91" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="24" t="inlineStr">
+        <is>
+          <t>IMP-21</t>
+        </is>
+      </c>
+      <c r="B92" s="24" t="inlineStr">
+        <is>
+          <t>Heat-Cool Portal</t>
+        </is>
+      </c>
+      <c r="C92" s="24" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="D92" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E92" s="24" t="inlineStr">
+        <is>
+          <t>Missing sorting functionality for the 'Recent Messages' table on the Building portal.</t>
+        </is>
+      </c>
+      <c r="F92" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A71:G71"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>